<commit_message>
update hayabusa return year
</commit_message>
<xml_diff>
--- a/tweetlist.xlsx
+++ b/tweetlist.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65AC2DB5-7AD1-4F8E-8054-6EA07361F2E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E987D207-271F-494E-9EC7-B9FD55F7582F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="885" yWindow="3840" windowWidth="14940" windowHeight="14955" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15" yWindow="4110" windowWidth="16200" windowHeight="18540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="todayssatellite" sheetId="1" r:id="rId1"/>
@@ -6872,26 +6872,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t xml:space="preserve">【お帰りはやぶさ・帰還15周年】6/9 12:30-15:00 最後の軌道修正となるTCM-4完了。4/4-6、5/1-4、5/23-27、6/3-5とあわせ5回の軌道修正でオーストラリア・ウーメラ砂漠の着陸地点へ誘導完了 </t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t xml:space="preserve">【お帰りはやぶさ・帰還15周年】6/13 19:54 イトカワのサンプルを格納したカプセルの切り離しに成功 </t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>【お帰りはやぶさ・帰還15周年】6/13 22:02 はやぶさ、最後の地球撮影。この写真 https://www.isas.jaxa.jp/j/topics/topics/2010/0618_3.shtml を内之浦局に送信中に内之浦の水平線の向こう側に入り通信途絶(22:28)</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t xml:space="preserve">【お帰りはやぶさ・帰還15周年】6/13 22:28 はやぶさ、内之浦局の観測圏外になり通信途絶。最後の信号はhttps://hayabusa.jaxa.jp/message/message_049.html に掲載されている </t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t xml:space="preserve">【お帰りはやぶさ・帰還15周年】6/13 22:51 はやぶさ、地球大気圏再突入。22:56にカプセルからパラシュートが展開され、23:08に着陸を果たした。 </t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>07/01 07:01:00</t>
     <phoneticPr fontId="1"/>
   </si>
@@ -7354,73 +7334,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>【お帰りはやぶさ2カプセル・帰還5周年】12/05 14:30 リュウグウのサンプルを格納したカプセルの切り離しに成功したことを確認</t>
-    <rPh sb="64" eb="66">
-      <t>カクニン</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>【お帰りはやぶさ2カプセル・帰還5周年】12/05 16:31 カプセル分離後、地球圏離脱のための軌道修正TCM-5の成功を確認。はやぶさ2は拡張ミッションへの軌道に乗り移った。</t>
-    <rPh sb="36" eb="39">
-      <t>ブンリゴ</t>
-    </rPh>
-    <rPh sb="40" eb="43">
-      <t>チキュウケン</t>
-    </rPh>
-    <rPh sb="43" eb="45">
-      <t>リダツ</t>
-    </rPh>
-    <rPh sb="49" eb="51">
-      <t>キドウ</t>
-    </rPh>
-    <rPh sb="51" eb="53">
-      <t>シュウセイ</t>
-    </rPh>
-    <rPh sb="59" eb="61">
-      <t>セイコウ</t>
-    </rPh>
-    <rPh sb="62" eb="64">
-      <t>カクニン</t>
-    </rPh>
-    <rPh sb="71" eb="73">
-      <t>カクチョウ</t>
-    </rPh>
-    <rPh sb="80" eb="82">
-      <t>キドウ</t>
-    </rPh>
-    <rPh sb="83" eb="84">
-      <t>ノ</t>
-    </rPh>
-    <rPh sb="85" eb="86">
-      <t>ウツ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t xml:space="preserve">【お帰りはやぶさ2カプセル・帰還5周年】12/06 02:54 はやぶさ2カプセル、ウーメラ砂漠に着陸を果たした。 </t>
-    <rPh sb="46" eb="48">
-      <t>サバク</t>
-    </rPh>
-    <rPh sb="49" eb="51">
-      <t>チャクリク</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>2025年版に修正</t>
-    <rPh sb="4" eb="5">
-      <t>ネン</t>
-    </rPh>
-    <rPh sb="5" eb="6">
-      <t>バン</t>
-    </rPh>
-    <rPh sb="7" eb="9">
-      <t>シュウセイ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>【今日の人工衛星】3/4 2010年：GOES-15 アメリカの気象観測衛星GOESのうちの1基。2011年より運用中だが、後継機のGOES-17が2018年に打ち上げられ、待機運用となったのち、2023年からは米宇宙軍の気象衛星EWS-G2として再活用されている。</t>
     <rPh sb="47" eb="48">
       <t>キ</t>
@@ -7655,6 +7568,93 @@
   </si>
   <si>
     <t>【今日の人工衛星】8/23(UTC)   2005年：れいめい   小型技術実証衛星。理学・工学ミッション以外に若手の技術習得も目的としていた。ながらく宇宙研から直接運用していたが、2025年7月に動作が停止、2026年3月4日に運用停止となった https://www.isas.jaxa.jp/topics/004204.html</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t xml:space="preserve">【お帰りはやぶさ・帰還17周年】6/9 12:30-15:00 最後の軌道修正となるTCM-4完了。4/4-6、5/1-4、5/23-27、6/3-5とあわせ5回の軌道修正でオーストラリア・ウーメラ砂漠の着陸地点へ誘導完了 </t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t xml:space="preserve">【お帰りはやぶさ・帰還16周年】6/13 19:54 イトカワのサンプルを格納したカプセルの切り離しに成功 </t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>【お帰りはやぶさ・帰還16周年】6/13 22:02 はやぶさ、最後の地球撮影。この写真 https://www.isas.jaxa.jp/j/topics/topics/2010/0618_3.shtml を内之浦局に送信中に内之浦の水平線の向こう側に入り通信途絶(22:28)</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t xml:space="preserve">【お帰りはやぶさ・帰還16周年】6/13 22:28 はやぶさ、内之浦局の観測圏外になり通信途絶。最後の信号はhttps://hayabusa.jaxa.jp/message/message_049.html に掲載されている </t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t xml:space="preserve">【お帰りはやぶさ・帰還16周年】6/13 22:51 はやぶさ、地球大気圏再突入。22:56にカプセルからパラシュートが展開され、23:08に着陸を果たした。 </t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>2026年版に修正</t>
+    <rPh sb="4" eb="5">
+      <t>ネン</t>
+    </rPh>
+    <rPh sb="5" eb="6">
+      <t>バン</t>
+    </rPh>
+    <rPh sb="7" eb="9">
+      <t>シュウセイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>【お帰りはやぶさ2カプセル・帰還6周年】12/05 14:30 リュウグウのサンプルを格納したカプセルの切り離しに成功したことを確認</t>
+    <rPh sb="64" eb="66">
+      <t>カクニン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>【お帰りはやぶさ2カプセル・帰還6周年】12/05 16:31 カプセル分離後、地球圏離脱のための軌道修正TCM-5の成功を確認。はやぶさ2は拡張ミッションへの軌道に乗り移った。</t>
+    <rPh sb="36" eb="39">
+      <t>ブンリゴ</t>
+    </rPh>
+    <rPh sb="40" eb="43">
+      <t>チキュウケン</t>
+    </rPh>
+    <rPh sb="43" eb="45">
+      <t>リダツ</t>
+    </rPh>
+    <rPh sb="49" eb="51">
+      <t>キドウ</t>
+    </rPh>
+    <rPh sb="51" eb="53">
+      <t>シュウセイ</t>
+    </rPh>
+    <rPh sb="59" eb="61">
+      <t>セイコウ</t>
+    </rPh>
+    <rPh sb="62" eb="64">
+      <t>カクニン</t>
+    </rPh>
+    <rPh sb="71" eb="73">
+      <t>カクチョウ</t>
+    </rPh>
+    <rPh sb="80" eb="82">
+      <t>キドウ</t>
+    </rPh>
+    <rPh sb="83" eb="84">
+      <t>ノ</t>
+    </rPh>
+    <rPh sb="85" eb="86">
+      <t>ウツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t xml:space="preserve">【お帰りはやぶさ2カプセル・帰還6周年】12/06 02:54 はやぶさ2カプセル、ウーメラ砂漠に着陸を果たした。 </t>
+    <rPh sb="46" eb="48">
+      <t>サバク</t>
+    </rPh>
+    <rPh sb="49" eb="51">
+      <t>チャクリク</t>
+    </rPh>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -14832,7 +14832,7 @@
         <v>504</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>1900</v>
+        <v>1891</v>
       </c>
       <c r="C37">
         <f t="shared" si="0"/>
@@ -14856,7 +14856,7 @@
         <v>20250620</v>
       </c>
       <c r="I37" t="s">
-        <v>1899</v>
+        <v>1890</v>
       </c>
     </row>
     <row r="38" spans="1:9" ht="27" x14ac:dyDescent="0.15">
@@ -15226,17 +15226,17 @@
     </row>
     <row r="53" spans="1:10" ht="27" x14ac:dyDescent="0.15">
       <c r="A53" s="1" t="s">
-        <v>1879</v>
+        <v>1874</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>1877</v>
+        <v>1872</v>
       </c>
       <c r="C53">
         <f t="shared" ref="C53:C54" si="2">LEN(B53)</f>
         <v>109</v>
       </c>
       <c r="D53" t="s">
-        <v>1875</v>
+        <v>1870</v>
       </c>
       <c r="E53" t="s">
         <v>1629</v>
@@ -15252,22 +15252,22 @@
         <v>20250202</v>
       </c>
       <c r="I53" t="s">
-        <v>1880</v>
+        <v>1875</v>
       </c>
     </row>
     <row r="54" spans="1:10" ht="27" x14ac:dyDescent="0.15">
       <c r="A54" s="1" t="s">
-        <v>1874</v>
+        <v>1869</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>1878</v>
+        <v>1873</v>
       </c>
       <c r="C54">
         <f t="shared" si="2"/>
         <v>119</v>
       </c>
       <c r="D54" t="s">
-        <v>1876</v>
+        <v>1871</v>
       </c>
       <c r="E54" t="s">
         <v>1629</v>
@@ -15283,7 +15283,7 @@
         <v>20250202</v>
       </c>
       <c r="I54" t="s">
-        <v>1880</v>
+        <v>1875</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.15">
@@ -17450,7 +17450,7 @@
         <v>596</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>1897</v>
+        <v>1888</v>
       </c>
       <c r="C139">
         <f t="shared" si="7"/>
@@ -17474,7 +17474,7 @@
         <v>1018</v>
       </c>
       <c r="J139" s="12" t="s">
-        <v>1898</v>
+        <v>1889</v>
       </c>
     </row>
     <row r="140" spans="1:10" ht="27" x14ac:dyDescent="0.15">
@@ -19339,7 +19339,7 @@
         <v>713</v>
       </c>
       <c r="B217" s="2" t="s">
-        <v>1848</v>
+        <v>1909</v>
       </c>
       <c r="C217">
         <f t="shared" si="9"/>
@@ -19359,7 +19359,7 @@
         <v>J_M5_5</v>
       </c>
       <c r="H217">
-        <v>20240614</v>
+        <v>20260611</v>
       </c>
       <c r="I217" t="s">
         <v>1004</v>
@@ -19370,7 +19370,7 @@
         <v>720</v>
       </c>
       <c r="B218" s="2" t="s">
-        <v>1849</v>
+        <v>1910</v>
       </c>
       <c r="C218">
         <f t="shared" si="9"/>
@@ -19390,7 +19390,7 @@
         <v>J_M5_5</v>
       </c>
       <c r="H218">
-        <v>20240614</v>
+        <v>20260611</v>
       </c>
       <c r="I218" t="s">
         <v>1004</v>
@@ -19401,7 +19401,7 @@
         <v>721</v>
       </c>
       <c r="B219" s="2" t="s">
-        <v>1850</v>
+        <v>1911</v>
       </c>
       <c r="C219">
         <f t="shared" si="9"/>
@@ -19421,7 +19421,7 @@
         <v>J_M5_5</v>
       </c>
       <c r="H219">
-        <v>20240614</v>
+        <v>20260611</v>
       </c>
       <c r="I219" t="s">
         <v>1004</v>
@@ -19432,7 +19432,7 @@
         <v>722</v>
       </c>
       <c r="B220" s="2" t="s">
-        <v>1851</v>
+        <v>1912</v>
       </c>
       <c r="C220">
         <f t="shared" si="9"/>
@@ -19452,7 +19452,7 @@
         <v>J_M5_5</v>
       </c>
       <c r="H220">
-        <v>20240614</v>
+        <v>20260611</v>
       </c>
       <c r="I220" t="s">
         <v>1004</v>
@@ -19463,7 +19463,7 @@
         <v>723</v>
       </c>
       <c r="B221" s="2" t="s">
-        <v>1852</v>
+        <v>1913</v>
       </c>
       <c r="C221">
         <f t="shared" si="9"/>
@@ -19483,7 +19483,7 @@
         <v>J_M5_5</v>
       </c>
       <c r="H221">
-        <v>20240614</v>
+        <v>20260611</v>
       </c>
       <c r="I221" t="s">
         <v>1004</v>
@@ -19747,7 +19747,7 @@
         <v>682</v>
       </c>
       <c r="B233" s="2" t="s">
-        <v>1909</v>
+        <v>1900</v>
       </c>
       <c r="C233">
         <f t="shared" si="9"/>
@@ -19856,7 +19856,7 @@
         <v>686</v>
       </c>
       <c r="B237" s="2" t="s">
-        <v>1910</v>
+        <v>1901</v>
       </c>
       <c r="C237">
         <f t="shared" si="9"/>
@@ -21131,20 +21131,20 @@
     </row>
     <row r="291" spans="1:10" ht="27" x14ac:dyDescent="0.15">
       <c r="A291" s="1" t="s">
-        <v>1907</v>
+        <v>1898</v>
       </c>
       <c r="B291" s="2" t="s">
-        <v>1908</v>
+        <v>1899</v>
       </c>
       <c r="C291">
         <f t="shared" si="11"/>
         <v>116</v>
       </c>
       <c r="D291" t="s">
-        <v>1901</v>
+        <v>1892</v>
       </c>
       <c r="E291" t="s">
-        <v>1903</v>
+        <v>1894</v>
       </c>
       <c r="F291">
         <v>50</v>
@@ -21157,25 +21157,25 @@
         <v>20250706</v>
       </c>
       <c r="I291" t="s">
-        <v>1904</v>
+        <v>1895</v>
       </c>
     </row>
     <row r="292" spans="1:10" ht="27" x14ac:dyDescent="0.15">
       <c r="A292" s="1" t="s">
-        <v>1906</v>
+        <v>1897</v>
       </c>
       <c r="B292" s="2" t="s">
-        <v>1911</v>
+        <v>1902</v>
       </c>
       <c r="C292">
         <f t="shared" si="11"/>
         <v>116</v>
       </c>
       <c r="D292" t="s">
-        <v>1902</v>
+        <v>1893</v>
       </c>
       <c r="E292" t="s">
-        <v>1903</v>
+        <v>1894</v>
       </c>
       <c r="F292">
         <v>50</v>
@@ -21191,7 +21191,7 @@
         <v>1004</v>
       </c>
       <c r="J292" t="s">
-        <v>1912</v>
+        <v>1903</v>
       </c>
     </row>
     <row r="293" spans="1:10" ht="27" x14ac:dyDescent="0.15">
@@ -21199,7 +21199,7 @@
         <v>743</v>
       </c>
       <c r="B293" s="2" t="s">
-        <v>1905</v>
+        <v>1896</v>
       </c>
       <c r="C293">
         <f t="shared" si="11"/>
@@ -21265,17 +21265,17 @@
     </row>
     <row r="296" spans="1:10" ht="27" x14ac:dyDescent="0.15">
       <c r="A296" s="1" t="s">
-        <v>1853</v>
+        <v>1848</v>
       </c>
       <c r="B296" s="2" t="s">
-        <v>1857</v>
+        <v>1852</v>
       </c>
       <c r="C296">
         <f t="shared" si="11"/>
         <v>110</v>
       </c>
       <c r="D296" t="s">
-        <v>1854</v>
+        <v>1849</v>
       </c>
       <c r="E296" t="s">
         <v>1629</v>
@@ -21290,17 +21290,17 @@
     </row>
     <row r="297" spans="1:10" ht="27" x14ac:dyDescent="0.15">
       <c r="A297" s="1" t="s">
-        <v>1856</v>
+        <v>1851</v>
       </c>
       <c r="B297" s="2" t="s">
-        <v>1858</v>
+        <v>1853</v>
       </c>
       <c r="C297">
         <f t="shared" si="11"/>
         <v>89</v>
       </c>
       <c r="D297" t="s">
-        <v>1855</v>
+        <v>1850</v>
       </c>
       <c r="E297" t="s">
         <v>1629</v>
@@ -21525,7 +21525,7 @@
         <v>755</v>
       </c>
       <c r="B307" s="2" t="s">
-        <v>1866</v>
+        <v>1861</v>
       </c>
       <c r="C307">
         <f t="shared" si="11"/>
@@ -21548,10 +21548,10 @@
         <v>20250129</v>
       </c>
       <c r="I307" t="s">
-        <v>1868</v>
+        <v>1863</v>
       </c>
       <c r="J307" t="s">
-        <v>1869</v>
+        <v>1864</v>
       </c>
     </row>
     <row r="308" spans="1:10" ht="27" x14ac:dyDescent="0.15">
@@ -21559,7 +21559,7 @@
         <v>756</v>
       </c>
       <c r="B308" s="2" t="s">
-        <v>1867</v>
+        <v>1862</v>
       </c>
       <c r="C308">
         <f t="shared" si="11"/>
@@ -21583,10 +21583,10 @@
         <v>20250129</v>
       </c>
       <c r="I308" t="s">
-        <v>1868</v>
+        <v>1863</v>
       </c>
       <c r="J308" t="s">
-        <v>1869</v>
+        <v>1864</v>
       </c>
     </row>
     <row r="309" spans="1:10" ht="27" x14ac:dyDescent="0.15">
@@ -23046,7 +23046,7 @@
         <v>818</v>
       </c>
       <c r="B369" s="2" t="s">
-        <v>1914</v>
+        <v>1905</v>
       </c>
       <c r="C369">
         <f t="shared" si="15"/>
@@ -23066,17 +23066,17 @@
     </row>
     <row r="370" spans="1:9" ht="40.5" x14ac:dyDescent="0.15">
       <c r="A370" s="1" t="s">
-        <v>1913</v>
+        <v>1904</v>
       </c>
       <c r="B370" s="2" t="s">
-        <v>1917</v>
+        <v>1908</v>
       </c>
       <c r="C370">
         <f t="shared" ref="C370" si="17">LEN(B370)</f>
         <v>167</v>
       </c>
       <c r="D370" t="s">
-        <v>1915</v>
+        <v>1906</v>
       </c>
       <c r="E370" t="str" cm="1">
         <f t="array" ref="E370">_xlfn.IFS(IFERROR(FIND("M-3SII",B370),-1)&gt;0,"J_M3S2",IFERROR(FIND("M-V",B370),-1)&gt;0,"J_M5",IFERROR(FIND("M-4S",B370),-1)&gt;0,"J_M4S",IFERROR(FIND("M-3C",B370),-1)&gt;0,"J_M3C",IFERROR(FIND("M-3S",B370),-1)&gt;0,"J_M3S",IFERROR(FIND("M-3H",B370),-1)&gt;0,"J_M3H",IFERROR(FIND("H-IIA",B370),-1)&gt;0,"J_H2A",IFERROR(FIND("H-IIB",B370),-1)&gt;0,"J_H2B",IFERROR(FIND("H-II",B370),-1)&gt;0,"J_H2",IFERROR(FIND("H-I",B370),-1)&gt;0,"J_H1",IFERROR(FIND("N-II",B370),-1)&gt;0,"J_N2",IFERROR(FIND("N-I",B370),-1)&gt;0,"J_N1",IFERROR(FIND("イプシロン",B370),-1)&gt;0,"J_E",TRUE,"")</f>
@@ -23090,7 +23090,7 @@
         <v>20260308</v>
       </c>
       <c r="I370" t="s">
-        <v>1916</v>
+        <v>1907</v>
       </c>
     </row>
     <row r="371" spans="1:9" ht="27" x14ac:dyDescent="0.15">
@@ -23808,17 +23808,17 @@
     </row>
     <row r="399" spans="1:9" ht="40.5" x14ac:dyDescent="0.15">
       <c r="A399" s="1" t="s">
-        <v>1859</v>
+        <v>1854</v>
       </c>
       <c r="B399" s="2" t="s">
-        <v>1860</v>
+        <v>1855</v>
       </c>
       <c r="C399">
         <f>LEN(B399)</f>
         <v>138</v>
       </c>
       <c r="D399" t="s">
-        <v>1863</v>
+        <v>1858</v>
       </c>
       <c r="E399" t="s">
         <v>1590</v>
@@ -23834,22 +23834,22 @@
         <v>20240826</v>
       </c>
       <c r="I399" t="s">
-        <v>1865</v>
+        <v>1860</v>
       </c>
     </row>
     <row r="400" spans="1:9" ht="27" x14ac:dyDescent="0.15">
       <c r="A400" s="1" t="s">
-        <v>1861</v>
+        <v>1856</v>
       </c>
       <c r="B400" s="2" t="s">
-        <v>1862</v>
+        <v>1857</v>
       </c>
       <c r="C400">
         <f>LEN(B400)</f>
         <v>78</v>
       </c>
       <c r="D400" t="s">
-        <v>1864</v>
+        <v>1859</v>
       </c>
       <c r="E400" t="str" cm="1">
         <f t="array" ref="E400">_xlfn.IFS(IFERROR(FIND("M-3SII",B400),-1)&gt;0,"J_M3S2",IFERROR(FIND("M-V",B400),-1)&gt;0,"J_M5",IFERROR(FIND("M-4S",B400),-1)&gt;0,"J_M4S",IFERROR(FIND("M-3C",B400),-1)&gt;0,"J_M3C",IFERROR(FIND("M-3S",B400),-1)&gt;0,"J_M3S",IFERROR(FIND("M-3H",B400),-1)&gt;0,"J_M3H",IFERROR(FIND("H-IIA",B400),-1)&gt;0,"J_H2A",IFERROR(FIND("H-IIB",B400),-1)&gt;0,"J_H2B",IFERROR(FIND("H-II",B400),-1)&gt;0,"J_H2",IFERROR(FIND("H-I",B400),-1)&gt;0,"J_H1",IFERROR(FIND("N-II",B400),-1)&gt;0,"J_N2",IFERROR(FIND("N-I",B400),-1)&gt;0,"J_N1",IFERROR(FIND("イプシロン",B400),-1)&gt;0,"J_E",TRUE,"")</f>
@@ -23866,7 +23866,7 @@
         <v>20240826</v>
       </c>
       <c r="I400" t="s">
-        <v>1865</v>
+        <v>1860</v>
       </c>
     </row>
     <row r="401" spans="1:9" ht="27" x14ac:dyDescent="0.15">
@@ -24782,17 +24782,17 @@
     </row>
     <row r="437" spans="1:9" ht="27" x14ac:dyDescent="0.15">
       <c r="A437" s="1" t="s">
-        <v>1887</v>
+        <v>1882</v>
       </c>
       <c r="B437" s="2" t="s">
-        <v>1889</v>
+        <v>1884</v>
       </c>
       <c r="C437">
         <f t="shared" ref="C437:C438" si="24">LEN(B437)</f>
         <v>105</v>
       </c>
       <c r="D437" t="s">
-        <v>1891</v>
+        <v>1886</v>
       </c>
       <c r="E437" t="str" cm="1">
         <f t="array" ref="E437">_xlfn.IFS(IFERROR(FIND("M-3SII",B437),-1)&gt;0,"J_M3S2",IFERROR(FIND("M-V",B437),-1)&gt;0,"J_M5",IFERROR(FIND("M-4S",B437),-1)&gt;0,"J_M4S",IFERROR(FIND("M-3C",B437),-1)&gt;0,"J_M3C",IFERROR(FIND("M-3S",B437),-1)&gt;0,"J_M3S",IFERROR(FIND("M-3H",B437),-1)&gt;0,"J_M3H",IFERROR(FIND("H-IIA",B437),-1)&gt;0,"J_H2A",IFERROR(FIND("H-IIB",B437),-1)&gt;0,"J_H2B",IFERROR(FIND("H-II",B437),-1)&gt;0,"J_H2",IFERROR(FIND("H-I",B437),-1)&gt;0,"J_H1",IFERROR(FIND("N-II",B437),-1)&gt;0,"J_N2",IFERROR(FIND("N-I",B437),-1)&gt;0,"J_N1",IFERROR(FIND("イプシロン",B437),-1)&gt;0,"J_E",TRUE,"")</f>
@@ -24814,17 +24814,17 @@
     </row>
     <row r="438" spans="1:9" ht="27" x14ac:dyDescent="0.15">
       <c r="A438" s="1" t="s">
-        <v>1888</v>
+        <v>1883</v>
       </c>
       <c r="B438" s="2" t="s">
-        <v>1890</v>
+        <v>1885</v>
       </c>
       <c r="C438">
         <f t="shared" si="24"/>
         <v>113</v>
       </c>
       <c r="D438" t="s">
-        <v>1892</v>
+        <v>1887</v>
       </c>
       <c r="E438" t="str" cm="1">
         <f t="array" ref="E438">_xlfn.IFS(IFERROR(FIND("M-3SII",B438),-1)&gt;0,"J_M3S2",IFERROR(FIND("M-V",B438),-1)&gt;0,"J_M5",IFERROR(FIND("M-4S",B438),-1)&gt;0,"J_M4S",IFERROR(FIND("M-3C",B438),-1)&gt;0,"J_M3C",IFERROR(FIND("M-3S",B438),-1)&gt;0,"J_M3S",IFERROR(FIND("M-3H",B438),-1)&gt;0,"J_M3H",IFERROR(FIND("H-IIA",B438),-1)&gt;0,"J_H2A",IFERROR(FIND("H-IIB",B438),-1)&gt;0,"J_H2B",IFERROR(FIND("H-II",B438),-1)&gt;0,"J_H2",IFERROR(FIND("H-I",B438),-1)&gt;0,"J_H1",IFERROR(FIND("N-II",B438),-1)&gt;0,"J_N2",IFERROR(FIND("N-I",B438),-1)&gt;0,"J_N1",IFERROR(FIND("イプシロン",B438),-1)&gt;0,"J_E",TRUE,"")</f>
@@ -25847,17 +25847,17 @@
     </row>
     <row r="482" spans="1:9" ht="27" x14ac:dyDescent="0.15">
       <c r="A482" s="1" t="s">
-        <v>1886</v>
+        <v>1881</v>
       </c>
       <c r="B482" s="2" t="s">
-        <v>1882</v>
+        <v>1877</v>
       </c>
       <c r="C482">
         <f t="shared" ref="C482:C483" si="28">LEN(B482)</f>
         <v>90</v>
       </c>
       <c r="D482" t="s">
-        <v>1884</v>
+        <v>1879</v>
       </c>
       <c r="E482" t="s">
         <v>1629</v>
@@ -25873,22 +25873,22 @@
         <v>20250202</v>
       </c>
       <c r="I482" t="s">
-        <v>1880</v>
+        <v>1875</v>
       </c>
     </row>
     <row r="483" spans="1:9" ht="27" x14ac:dyDescent="0.15">
       <c r="A483" s="1" t="s">
-        <v>1881</v>
+        <v>1876</v>
       </c>
       <c r="B483" s="2" t="s">
-        <v>1883</v>
+        <v>1878</v>
       </c>
       <c r="C483">
         <f t="shared" si="28"/>
         <v>100</v>
       </c>
       <c r="D483" t="s">
-        <v>1885</v>
+        <v>1880</v>
       </c>
       <c r="E483" t="s">
         <v>1629</v>
@@ -25904,7 +25904,7 @@
         <v>20250202</v>
       </c>
       <c r="I483" t="s">
-        <v>1880</v>
+        <v>1875</v>
       </c>
     </row>
     <row r="484" spans="1:9" ht="27" x14ac:dyDescent="0.15">
@@ -26824,7 +26824,7 @@
         <v>1034</v>
       </c>
       <c r="B521" s="2" t="s">
-        <v>1893</v>
+        <v>1915</v>
       </c>
       <c r="C521">
         <f t="shared" si="26"/>
@@ -26844,13 +26844,13 @@
         <v>J_H2A_26</v>
       </c>
       <c r="H521">
-        <v>20250202</v>
+        <v>20260611</v>
       </c>
       <c r="I521" t="s">
         <v>1004</v>
       </c>
       <c r="J521" t="s">
-        <v>1896</v>
+        <v>1914</v>
       </c>
     </row>
     <row r="522" spans="1:11" ht="27" x14ac:dyDescent="0.15">
@@ -26858,7 +26858,7 @@
         <v>1035</v>
       </c>
       <c r="B522" s="2" t="s">
-        <v>1894</v>
+        <v>1916</v>
       </c>
       <c r="C522">
         <f t="shared" si="26"/>
@@ -26878,13 +26878,13 @@
         <v>J_H2A_26</v>
       </c>
       <c r="H522">
-        <v>20250202</v>
+        <v>20260611</v>
       </c>
       <c r="I522" t="s">
         <v>1004</v>
       </c>
       <c r="J522" t="s">
-        <v>1896</v>
+        <v>1914</v>
       </c>
     </row>
     <row r="523" spans="1:11" x14ac:dyDescent="0.15">
@@ -26892,7 +26892,7 @@
         <v>1033</v>
       </c>
       <c r="B523" s="2" t="s">
-        <v>1895</v>
+        <v>1917</v>
       </c>
       <c r="C523">
         <f t="shared" si="26"/>
@@ -26912,13 +26912,13 @@
         <v>J_H2A_26</v>
       </c>
       <c r="H523">
-        <v>20250202</v>
+        <v>20260611</v>
       </c>
       <c r="I523" t="s">
         <v>1004</v>
       </c>
       <c r="J523" t="s">
-        <v>1896</v>
+        <v>1914</v>
       </c>
     </row>
     <row r="524" spans="1:11" ht="27" x14ac:dyDescent="0.15">
@@ -27792,7 +27792,7 @@
         <v>989</v>
       </c>
       <c r="B560" s="2" t="s">
-        <v>1872</v>
+        <v>1867</v>
       </c>
       <c r="C560">
         <f t="shared" si="31"/>
@@ -27813,10 +27813,10 @@
         <v>20250129</v>
       </c>
       <c r="I560" t="s">
-        <v>1871</v>
+        <v>1866</v>
       </c>
       <c r="J560" t="s">
-        <v>1870</v>
+        <v>1865</v>
       </c>
     </row>
     <row r="561" spans="1:2" x14ac:dyDescent="0.15">
@@ -31590,7 +31590,7 @@
     </row>
     <row r="98" spans="2:17" x14ac:dyDescent="0.15">
       <c r="B98" s="5" t="s">
-        <v>1873</v>
+        <v>1868</v>
       </c>
       <c r="C98" s="5">
         <v>4</v>
@@ -31617,7 +31617,7 @@
     </row>
     <row r="99" spans="2:17" x14ac:dyDescent="0.15">
       <c r="B99" s="5" t="s">
-        <v>1873</v>
+        <v>1868</v>
       </c>
       <c r="C99" s="5">
         <v>5</v>
@@ -31644,7 +31644,7 @@
     </row>
     <row r="100" spans="2:17" x14ac:dyDescent="0.15">
       <c r="B100" s="5" t="s">
-        <v>1873</v>
+        <v>1868</v>
       </c>
       <c r="C100" s="5">
         <v>6</v>

</xml_diff>